<commit_message>
avoided cost final reset
</commit_message>
<xml_diff>
--- a/00_input/00_Potential_Study_Input_Template.xlsx
+++ b/00_input/00_Potential_Study_Input_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nv5inc-my.sharepoint.com/personal/andrewj_johnson_nv5_com/Documents/Documents/GitHub/Potential_Study_Tool_Prototype/00_input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="107" documentId="11_A19FC89F29AA3734ADFF971C77E100913CED4083" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{357FED74-70F8-42D5-AA41-D22187DB650B}"/>
+  <xr:revisionPtr revIDLastSave="120" documentId="11_A19FC89F29AA3734ADFF971C77E100913CED4083" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74576ABC-CA1F-4CCE-B929-17402A8BDB04}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-3420" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-3420" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Measure_List" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="75">
   <si>
     <t>Measure Name</t>
   </si>
@@ -90,18 +90,12 @@
     <t>natural gas</t>
   </si>
   <si>
-    <t>central_ac</t>
-  </si>
-  <si>
     <t>MD</t>
   </si>
   <si>
     <t>electric</t>
   </si>
   <si>
-    <t>room_ac</t>
-  </si>
-  <si>
     <t>fridge</t>
   </si>
   <si>
@@ -120,60 +114,6 @@
     <t>Multifamily LI</t>
   </si>
   <si>
-    <t>Large Restaurant</t>
-  </si>
-  <si>
-    <t>Large Hospital</t>
-  </si>
-  <si>
-    <t>Large Hotel</t>
-  </si>
-  <si>
-    <t>Large Office</t>
-  </si>
-  <si>
-    <t>Large Outpatient</t>
-  </si>
-  <si>
-    <t>Large Primary secondary school</t>
-  </si>
-  <si>
-    <t>Large Retail</t>
-  </si>
-  <si>
-    <t>Large Strip mall</t>
-  </si>
-  <si>
-    <t>Large Warehouse</t>
-  </si>
-  <si>
-    <t>Small Restaurant</t>
-  </si>
-  <si>
-    <t>Small Hospital</t>
-  </si>
-  <si>
-    <t>Small Hotel</t>
-  </si>
-  <si>
-    <t>Small Office</t>
-  </si>
-  <si>
-    <t>Small Outpatient</t>
-  </si>
-  <si>
-    <t>Small Primary secondary school</t>
-  </si>
-  <si>
-    <t>Small Retail</t>
-  </si>
-  <si>
-    <t>Small Strip mall</t>
-  </si>
-  <si>
-    <t>Small Warehouse</t>
-  </si>
-  <si>
     <t>Screening Data</t>
   </si>
   <si>
@@ -234,9 +174,6 @@
     <t>efficiency_levels</t>
   </si>
   <si>
-    <t>Ret_add_on</t>
-  </si>
-  <si>
     <t>competition_group</t>
   </si>
   <si>
@@ -250,9 +187,6 @@
   </si>
   <si>
     <t>gas_furnace</t>
-  </si>
-  <si>
-    <t>cooling</t>
   </si>
   <si>
     <t>refrigeration</t>
@@ -826,10 +760,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" customWidth="1"/>
+    <col min="5" max="5" width="21.42578125" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -843,16 +781,16 @@
         <v>2</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -869,13 +807,13 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>59</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -892,151 +830,59 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" t="s">
-        <v>55</v>
-      </c>
-      <c r="C7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8">
-        <v>2</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9">
-        <v>2</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="G9" s="9" t="s">
-        <v>63</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1047,7 +893,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82018058-B319-44E1-8463-34F498BF93D1}">
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.140625" customWidth="1"/>
@@ -1055,117 +901,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1175,7 +931,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F87D81C9-F45F-4EDB-B264-48D1BD0F9B8E}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -1184,67 +940,47 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>66</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>67</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>68</v>
-      </c>
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>68</v>
-      </c>
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>67</v>
-      </c>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1255,70 +991,73 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB87DCD5-5DFC-46FE-AE66-5108DCD2E4AE}">
   <dimension ref="A1:A13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>84</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>85</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>88</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>89</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>91</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>92</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>95</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>96</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1333,57 +1072,57 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>73</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>74</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>75</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>76</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>77</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>78</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>79</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>83</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>80</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>81</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>82</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
@@ -1405,16 +1144,16 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="C1" s="2"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="B2" s="4">
         <v>2026</v>
@@ -1423,45 +1162,45 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="B3" s="4">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="B5" s="5">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="B6" s="5">
         <v>1.9417500000000001E-2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="B7" s="6">
         <v>2026</v>
@@ -1469,7 +1208,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="B8" s="7">
         <f>B2</f>
@@ -1479,13 +1218,13 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="B9" s="8">
         <v>0.02</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1493,51 +1232,51 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>47</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="B12" s="5">
         <v>2.999997547619106E-2</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="B13" s="5">
         <v>2.999997547619106E-2</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="B14" s="5">
         <v>2.999997547619106E-2</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="B15" s="5">
         <v>2.999997547619106E-2</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1558,22 +1297,22 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>69</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>70</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
puh of major updates
</commit_message>
<xml_diff>
--- a/00_input/00_Potential_Study_Input_Template.xlsx
+++ b/00_input/00_Potential_Study_Input_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nv5inc-my.sharepoint.com/personal/andrewj_johnson_nv5_com/Documents/Documents/GitHub/Potential_Study_Tool_Prototype/00_input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="123" documentId="11_A19FC89F29AA3734ADFF971C77E100913CED4083" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7A13A48-8A89-4687-B2E6-2A6BFB512CF1}"/>
+  <xr:revisionPtr revIDLastSave="124" documentId="11_A19FC89F29AA3734ADFF971C77E100913CED4083" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E99E9DB4-5FCF-475E-B4E2-D1A853EC8A98}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="60795" yWindow="-525" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Measure_List" sheetId="1" r:id="rId1"/>
@@ -768,6 +768,7 @@
     <col min="4" max="4" width="18.5703125" customWidth="1"/>
     <col min="5" max="5" width="21.42578125" customWidth="1"/>
     <col min="6" max="6" width="18.28515625" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1321,12 +1322,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B011C3FEFFEFCF44990405A8404263A2" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ff8dfd3bc83a02ed6a3437faf473449a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79a1cdf2-2d4f-42d7-aee4-ff0e208e0f4a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8a600ae29b0fcdec2bdff655f54bd0a0" ns2:_="">
     <xsd:import namespace="79a1cdf2-2d4f-42d7-aee4-ff0e208e0f4a"/>
@@ -1470,6 +1465,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1480,15 +1481,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A32039BA-EC30-45DE-8DE0-801CC83D07E3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D903FE06-E673-438D-9976-4DA8E45A8B2B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1506,6 +1498,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A32039BA-EC30-45DE-8DE0-801CC83D07E3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2C5716C-2B48-488E-8F5B-6FDC8A1B108E}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
updates to template work
</commit_message>
<xml_diff>
--- a/00_input/00_Potential_Study_Input_Template.xlsx
+++ b/00_input/00_Potential_Study_Input_Template.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nv5inc-my.sharepoint.com/personal/andrewj_johnson_nv5_com/Documents/Documents/GitHub/Potential_Study_Tool_Prototype/00_input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="124" documentId="11_A19FC89F29AA3734ADFF971C77E100913CED4083" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E99E9DB4-5FCF-475E-B4E2-D1A853EC8A98}"/>
+  <xr:revisionPtr revIDLastSave="134" documentId="11_A19FC89F29AA3734ADFF971C77E100913CED4083" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48D8B0A2-A91C-468A-8B23-045DBE40EB63}"/>
   <bookViews>
-    <workbookView xWindow="60795" yWindow="-525" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Measure_List" sheetId="1" r:id="rId1"/>
-    <sheet name="Building_Types" sheetId="2" r:id="rId2"/>
-    <sheet name="Utility_Combinations" sheetId="3" r:id="rId3"/>
+    <sheet name="Global_Inputs" sheetId="7" r:id="rId1"/>
+    <sheet name="Measure_List" sheetId="1" r:id="rId2"/>
+    <sheet name="Building_Types" sheetId="2" r:id="rId3"/>
     <sheet name="Programs" sheetId="4" r:id="rId4"/>
     <sheet name="Periods" sheetId="5" r:id="rId5"/>
     <sheet name="ghgs" sheetId="8" r:id="rId6"/>
-    <sheet name="Global_Inputs" sheetId="7" r:id="rId7"/>
+    <sheet name="Utility_Combinations" sheetId="3" r:id="rId7"/>
+    <sheet name="vocabulary_enums" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -67,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="77">
   <si>
     <t>Measure Name</t>
   </si>
@@ -292,6 +293,12 @@
   </si>
   <si>
     <t>refrigerator</t>
+  </si>
+  <si>
+    <t>Characterization Unit</t>
+  </si>
+  <si>
+    <t>widget</t>
   </si>
 </sst>
 </file>
@@ -759,8 +766,165 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18CE5995-339E-40D5-B166-EF3D0F0BBE56}">
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="4">
+        <v>2026</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="4">
+        <v>20</v>
+      </c>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="5">
+        <v>0.03</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="5">
+        <v>1.9417500000000001E-2</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="6">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="7">
+        <f>B2</f>
+        <v>2026</v>
+      </c>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="8">
+        <v>0.02</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="5">
+        <v>2.999997547619106E-2</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="5">
+        <v>2.999997547619106E-2</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="5">
+        <v>2.999997547619106E-2</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="5">
+        <v>2.999997547619106E-2</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B9 B5:B6 B12:B15" xr:uid="{25FC0D5C-5FFE-4972-852D-3A9C7643127A}">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.85546875" customWidth="1"/>
@@ -771,7 +935,7 @@
     <col min="7" max="7" width="12.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -793,8 +957,11 @@
       <c r="G1" s="9" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -816,8 +983,11 @@
       <c r="G2" s="9" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" s="9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -839,8 +1009,11 @@
       <c r="G3" s="9" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" s="9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>74</v>
       </c>
@@ -862,8 +1035,11 @@
       <c r="G4" s="9" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" s="9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>74</v>
       </c>
@@ -884,6 +1060,9 @@
       </c>
       <c r="G5" s="9" t="s">
         <v>40</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -892,7 +1071,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82018058-B319-44E1-8463-34F498BF93D1}">
   <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -930,7 +1109,183 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB87DCD5-5DFC-46FE-AE66-5108DCD2E4AE}">
+  <dimension ref="A1:A13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF8172CC-7EBC-4E99-93A4-7009471032A9}">
+  <dimension ref="A1:A12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="9"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A95EC045-8ABC-4990-9ABC-9618212FDF50}">
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F87D81C9-F45F-4EDB-B264-48D1BD0F9B8E}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -988,335 +1343,11 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB87DCD5-5DFC-46FE-AE66-5108DCD2E4AE}">
-  <dimension ref="A1:A13"/>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DFD0B07-4704-4148-A894-77EA41CDECAA}">
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="13.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>73</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF8172CC-7EBC-4E99-93A4-7009471032A9}">
-  <dimension ref="A1:A12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A95EC045-8ABC-4990-9ABC-9618212FDF50}">
-  <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
-        <v>49</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18CE5995-339E-40D5-B166-EF3D0F0BBE56}">
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="30.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="2"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="4">
-        <v>2026</v>
-      </c>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="4">
-        <v>20</v>
-      </c>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="5">
-        <v>0.03</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" s="5">
-        <v>1.9417500000000001E-2</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="6">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="7">
-        <f>B2</f>
-        <v>2026</v>
-      </c>
-      <c r="C8" s="2"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="8">
-        <v>0.02</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="5">
-        <v>2.999997547619106E-2</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="5">
-        <v>2.999997547619106E-2</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14" s="5">
-        <v>2.999997547619106E-2</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="5">
-        <v>2.999997547619106E-2</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B9 B5:B6 B12:B15" xr:uid="{25FC0D5C-5FFE-4972-852D-3A9C7643127A}">
-      <formula1>0</formula1>
-      <formula2>1</formula2>
-    </dataValidation>
-  </dataValidations>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
edits to climate zone and secondary savings flag plan
</commit_message>
<xml_diff>
--- a/00_input/00_Potential_Study_Input_Template.xlsx
+++ b/00_input/00_Potential_Study_Input_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nv5inc-my.sharepoint.com/personal/andrewj_johnson_nv5_com/Documents/Documents/GitHub/Potential_Study_Tool_Prototype/00_input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="180" documentId="11_A19FC89F29AA3734ADFF971C77E100913CED4083" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF9BC213-157A-4FFD-A3F8-E1B4670AB643}"/>
+  <xr:revisionPtr revIDLastSave="186" documentId="11_A19FC89F29AA3734ADFF971C77E100913CED4083" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8A277C0-A57C-4910-9C5F-50FD84EFE961}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1890" yWindow="3405" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global_Inputs" sheetId="7" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="97">
   <si>
     <t>Measure Name</t>
   </si>
@@ -350,6 +350,15 @@
   </si>
   <si>
     <t>climate_zone</t>
+  </si>
+  <si>
+    <t>climate_zone_relevance</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>n</t>
   </si>
 </sst>
 </file>
@@ -468,7 +477,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -499,9 +508,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -983,7 +989,7 @@
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="3" t="s">
         <v>92</v>
       </c>
     </row>
@@ -1000,7 +1006,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.85546875" customWidth="1"/>
@@ -1011,14 +1017,14 @@
     <col min="7" max="7" width="12.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="12" t="s">
         <v>90</v>
       </c>
       <c r="D1" s="10" t="s">
@@ -1036,8 +1042,11 @@
       <c r="H1" s="10" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1062,8 +1071,11 @@
       <c r="H2" s="9" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1088,8 +1100,11 @@
       <c r="H3" s="9" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>70</v>
       </c>
@@ -1114,8 +1129,11 @@
       <c r="H4" s="9" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I4" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>70</v>
       </c>
@@ -1139,6 +1157,9 @@
       </c>
       <c r="H5" s="9" t="s">
         <v>71</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1400,7 +1421,7 @@
         <v>41</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1649,18 +1670,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1682,18 +1703,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2C5716C-2B48-488E-8F5B-6FDC8A1B108E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A32039BA-EC30-45DE-8DE0-801CC83D07E3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2C5716C-2B48-488E-8F5B-6FDC8A1B108E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add feasibility constraints and input sheet generation
Introduces feasibility constraints to the adoption model by adding a 'feasibility_constraint' column to relevant dataframes and generating a new 35_Feasibility_Inputs.xlsx workbook. Updates the template creation notebook to filter and export feasible measures, and documents the feature in a new PRD. All relevant input and output templates are updated to support this new constraint mechanism.
</commit_message>
<xml_diff>
--- a/00_input/00_Potential_Study_Input_Template.xlsx
+++ b/00_input/00_Potential_Study_Input_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nv5inc-my.sharepoint.com/personal/andrewj_johnson_nv5_com/Documents/Documents/GitHub/Potential_Study_Tool_Prototype/00_input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="186" documentId="11_A19FC89F29AA3734ADFF971C77E100913CED4083" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8A277C0-A57C-4910-9C5F-50FD84EFE961}"/>
+  <xr:revisionPtr revIDLastSave="195" documentId="11_A19FC89F29AA3734ADFF971C77E100913CED4083" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E5CEC72-FD07-46E7-A35F-E8BDCD236469}"/>
   <bookViews>
-    <workbookView xWindow="1890" yWindow="3405" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-3420" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global_Inputs" sheetId="7" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="98">
   <si>
     <t>Measure Name</t>
   </si>
@@ -359,6 +359,9 @@
   </si>
   <si>
     <t>n</t>
+  </si>
+  <si>
+    <t>feasibility_constraint</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +1009,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.85546875" customWidth="1"/>
@@ -1015,9 +1018,10 @@
     <col min="5" max="5" width="21.42578125" customWidth="1"/>
     <col min="6" max="6" width="18.28515625" customWidth="1"/>
     <col min="7" max="7" width="12.140625" customWidth="1"/>
+    <col min="9" max="9" width="25.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -1045,8 +1049,11 @@
       <c r="I1" s="10" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" s="12" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1074,8 +1081,11 @@
       <c r="I2" s="9" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J2" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1103,8 +1113,11 @@
       <c r="I3" s="9" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J3" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>70</v>
       </c>
@@ -1132,8 +1145,11 @@
       <c r="I4" s="9" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J4" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>70</v>
       </c>
@@ -1161,8 +1177,16 @@
       <c r="I5" s="9" t="s">
         <v>96</v>
       </c>
+      <c r="J5" s="9" t="s">
+        <v>95</v>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:J27" xr:uid="{C2276F6B-D3FD-47F4-90ED-57E44A2C1899}">
+      <formula1>"y,n"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
@@ -1526,6 +1550,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B011C3FEFFEFCF44990405A8404263A2" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ff8dfd3bc83a02ed6a3437faf473449a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79a1cdf2-2d4f-42d7-aee4-ff0e208e0f4a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8a600ae29b0fcdec2bdff655f54bd0a0" ns2:_="">
     <xsd:import namespace="79a1cdf2-2d4f-42d7-aee4-ff0e208e0f4a"/>
@@ -1669,22 +1708,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A32039BA-EC30-45DE-8DE0-801CC83D07E3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2C5716C-2B48-488E-8F5B-6FDC8A1B108E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D903FE06-E673-438D-9976-4DA8E45A8B2B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1700,21 +1741,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2C5716C-2B48-488E-8F5B-6FDC8A1B108E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A32039BA-EC30-45DE-8DE0-801CC83D07E3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>